<commit_message>
Confirm 135 dates from Umut iphone cell stocks
</commit_message>
<xml_diff>
--- a/cellstocks/cell-stocks.xlsx
+++ b/cellstocks/cell-stocks.xlsx
@@ -184,14 +184,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-05-05</t>
+        </is>
+      </c>
       <c r="I2" t="inlineStr">
         <is>
           <t xml:space="preserve">5/5/2025</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -266,14 +266,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-05-05</t>
+        </is>
+      </c>
       <c r="I3" t="inlineStr">
         <is>
           <t xml:space="preserve">5/5/2025</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -348,14 +348,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-05-05</t>
+        </is>
+      </c>
       <c r="I4" t="inlineStr">
         <is>
           <t xml:space="preserve">5/5/2025</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -430,14 +430,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-05-05</t>
+        </is>
+      </c>
       <c r="I5" t="inlineStr">
         <is>
           <t xml:space="preserve">5/5/2025</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -512,14 +512,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-04-09</t>
+        </is>
+      </c>
       <c r="I6" t="inlineStr">
         <is>
           <t xml:space="preserve">9/4/2026</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -594,14 +594,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-04-09</t>
+        </is>
+      </c>
       <c r="I7" t="inlineStr">
         <is>
           <t xml:space="preserve">9/4/2026</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -840,14 +840,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-02-10</t>
+        </is>
+      </c>
       <c r="I10" t="inlineStr">
         <is>
           <t xml:space="preserve">10/2/2026</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1578,14 +1578,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-05-08</t>
+        </is>
+      </c>
       <c r="I19" t="inlineStr">
         <is>
           <t xml:space="preserve">8/5/2025</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -1660,14 +1660,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-05-08</t>
+        </is>
+      </c>
       <c r="I20" t="inlineStr">
         <is>
           <t xml:space="preserve">8/5/2025</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -1742,14 +1742,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-05-08</t>
+        </is>
+      </c>
       <c r="I21" t="inlineStr">
         <is>
           <t xml:space="preserve">8/5/2025</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1824,14 +1824,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-05-08</t>
+        </is>
+      </c>
       <c r="I22" t="inlineStr">
         <is>
           <t xml:space="preserve">8/5/2025</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1906,14 +1906,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-05-07</t>
+        </is>
+      </c>
       <c r="I23" t="inlineStr">
         <is>
           <t xml:space="preserve">7/5/2025</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -1988,14 +1988,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-05-07</t>
+        </is>
+      </c>
       <c r="I24" t="inlineStr">
         <is>
           <t xml:space="preserve">7/5/2025</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -2070,14 +2070,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-05-07</t>
+        </is>
+      </c>
       <c r="I25" t="inlineStr">
         <is>
           <t xml:space="preserve">7/5/2025</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -3176,14 +3176,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023-02-03</t>
+        </is>
+      </c>
       <c r="I38" t="inlineStr">
         <is>
           <t xml:space="preserve">3/2/2023</t>
-        </is>
-      </c>
-      <c r="J38" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -3340,14 +3340,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-05-02</t>
+        </is>
+      </c>
       <c r="I40" t="inlineStr">
         <is>
           <t xml:space="preserve">2/5/2025</t>
-        </is>
-      </c>
-      <c r="J40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -3750,14 +3750,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-02-06</t>
+        </is>
+      </c>
       <c r="I45" t="inlineStr">
         <is>
           <t xml:space="preserve">6/2/2026</t>
-        </is>
-      </c>
-      <c r="J45" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -3914,14 +3914,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-02-05</t>
+        </is>
+      </c>
       <c r="I47" t="inlineStr">
         <is>
           <t xml:space="preserve">5/2/2026</t>
-        </is>
-      </c>
-      <c r="J47" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
@@ -3996,14 +3996,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-02-02</t>
+        </is>
+      </c>
       <c r="I48" t="inlineStr">
         <is>
           <t xml:space="preserve">2/2/2026</t>
-        </is>
-      </c>
-      <c r="J48" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
@@ -4160,14 +4160,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-02-02</t>
+        </is>
+      </c>
       <c r="I50" t="inlineStr">
         <is>
           <t xml:space="preserve">2/2/2026</t>
-        </is>
-      </c>
-      <c r="J50" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
@@ -4324,14 +4324,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-03</t>
+        </is>
+      </c>
       <c r="I52" t="inlineStr">
         <is>
           <t xml:space="preserve">3/3/2026</t>
-        </is>
-      </c>
-      <c r="J52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
@@ -4406,14 +4406,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-03</t>
+        </is>
+      </c>
       <c r="I53" t="inlineStr">
         <is>
           <t xml:space="preserve">3/3/2026</t>
-        </is>
-      </c>
-      <c r="J53" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -5686,14 +5686,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-02-02</t>
+        </is>
+      </c>
       <c r="I68" t="inlineStr">
         <is>
           <t xml:space="preserve">2/2/2026</t>
-        </is>
-      </c>
-      <c r="J68" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
@@ -5850,14 +5850,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-02-02</t>
+        </is>
+      </c>
       <c r="I70" t="inlineStr">
         <is>
           <t xml:space="preserve">2/2/2026</t>
-        </is>
-      </c>
-      <c r="J70" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
@@ -6096,14 +6096,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-04-10</t>
+        </is>
+      </c>
       <c r="I73" t="inlineStr">
         <is>
           <t xml:space="preserve">10/4/2026</t>
-        </is>
-      </c>
-      <c r="J73" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
@@ -6178,14 +6178,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-04-10</t>
+        </is>
+      </c>
       <c r="I74" t="inlineStr">
         <is>
           <t xml:space="preserve">10/4/2026</t>
-        </is>
-      </c>
-      <c r="J74" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
@@ -6834,14 +6834,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-10</t>
+        </is>
+      </c>
       <c r="I82" t="inlineStr">
         <is>
           <t xml:space="preserve">10/3/2026</t>
-        </is>
-      </c>
-      <c r="J82" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K82" t="inlineStr">
@@ -6916,14 +6916,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-11</t>
+        </is>
+      </c>
       <c r="I83" t="inlineStr">
         <is>
           <t xml:space="preserve">11/3/2026</t>
-        </is>
-      </c>
-      <c r="J83" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K83" t="inlineStr">
@@ -6998,14 +6998,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-11</t>
+        </is>
+      </c>
       <c r="I84" t="inlineStr">
         <is>
           <t xml:space="preserve">11/3/2026</t>
-        </is>
-      </c>
-      <c r="J84" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K84" t="inlineStr">
@@ -7080,14 +7080,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-10</t>
+        </is>
+      </c>
       <c r="I85" t="inlineStr">
         <is>
           <t xml:space="preserve">10/3/2026</t>
-        </is>
-      </c>
-      <c r="J85" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K85" t="inlineStr">
@@ -7244,14 +7244,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-07-07</t>
+        </is>
+      </c>
       <c r="I87" t="inlineStr">
         <is>
           <t xml:space="preserve">7/7/2025</t>
-        </is>
-      </c>
-      <c r="J87" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K87" t="inlineStr">
@@ -7336,14 +7336,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-06-09</t>
+        </is>
+      </c>
       <c r="I88" t="inlineStr">
         <is>
           <t xml:space="preserve">9/6/2026</t>
-        </is>
-      </c>
-      <c r="J88" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">
@@ -7500,14 +7500,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-06-09</t>
+        </is>
+      </c>
       <c r="I90" t="inlineStr">
         <is>
           <t xml:space="preserve">9/6/2026</t>
-        </is>
-      </c>
-      <c r="J90" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K90" t="inlineStr">
@@ -7582,14 +7582,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-05-08</t>
+        </is>
+      </c>
       <c r="I91" t="inlineStr">
         <is>
           <t xml:space="preserve">8/5/2026</t>
-        </is>
-      </c>
-      <c r="J91" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K91" t="inlineStr">
@@ -8402,14 +8402,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-11-10</t>
+        </is>
+      </c>
       <c r="I101" t="inlineStr">
         <is>
           <t xml:space="preserve">10/11/2025</t>
-        </is>
-      </c>
-      <c r="J101" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K101" t="inlineStr">
@@ -8484,14 +8484,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-11-10</t>
+        </is>
+      </c>
       <c r="I102" t="inlineStr">
         <is>
           <t xml:space="preserve">10/11/2025</t>
-        </is>
-      </c>
-      <c r="J102" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K102" t="inlineStr">
@@ -8566,14 +8566,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-06-02</t>
+        </is>
+      </c>
       <c r="I103" t="inlineStr">
         <is>
           <t xml:space="preserve">2/6/2025</t>
-        </is>
-      </c>
-      <c r="J103" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K103" t="inlineStr">
@@ -8658,14 +8658,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-05-08</t>
+        </is>
+      </c>
       <c r="I104" t="inlineStr">
         <is>
           <t xml:space="preserve">8/5/2026</t>
-        </is>
-      </c>
-      <c r="J104" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K104" t="inlineStr">
@@ -8822,14 +8822,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-10-09</t>
+        </is>
+      </c>
       <c r="I106" t="inlineStr">
         <is>
           <t xml:space="preserve">9/10/2025</t>
-        </is>
-      </c>
-      <c r="J106" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K106" t="inlineStr">
@@ -8904,14 +8904,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-10-09</t>
+        </is>
+      </c>
       <c r="I107" t="inlineStr">
         <is>
           <t xml:space="preserve">9/10/2025</t>
-        </is>
-      </c>
-      <c r="J107" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K107" t="inlineStr">
@@ -8986,14 +8986,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-10-09</t>
+        </is>
+      </c>
       <c r="I108" t="inlineStr">
         <is>
           <t xml:space="preserve">9/10/2025</t>
-        </is>
-      </c>
-      <c r="J108" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K108" t="inlineStr">
@@ -9396,14 +9396,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-05-06</t>
+        </is>
+      </c>
       <c r="I113" t="inlineStr">
         <is>
           <t xml:space="preserve">6/5/2026</t>
-        </is>
-      </c>
-      <c r="J113" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K113" t="inlineStr">
@@ -9478,14 +9478,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-05-06</t>
+        </is>
+      </c>
       <c r="I114" t="inlineStr">
         <is>
           <t xml:space="preserve">6/5/2026</t>
-        </is>
-      </c>
-      <c r="J114" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K114" t="inlineStr">
@@ -9724,14 +9724,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-01-06</t>
+        </is>
+      </c>
       <c r="I117" t="inlineStr">
         <is>
           <t xml:space="preserve">6/1/2025</t>
-        </is>
-      </c>
-      <c r="J117" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -10298,14 +10298,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-12-05</t>
+        </is>
+      </c>
       <c r="I124" t="inlineStr">
         <is>
           <t xml:space="preserve">5/12/2025</t>
-        </is>
-      </c>
-      <c r="J124" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K124" t="inlineStr">
@@ -10380,14 +10380,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-12-11</t>
+        </is>
+      </c>
       <c r="I125" t="inlineStr">
         <is>
           <t xml:space="preserve">11/12/2025</t>
-        </is>
-      </c>
-      <c r="J125" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K125" t="inlineStr">
@@ -10462,14 +10462,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-10-07</t>
+        </is>
+      </c>
       <c r="I126" t="inlineStr">
         <is>
           <t xml:space="preserve">7/10/2025</t>
-        </is>
-      </c>
-      <c r="J126" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K126" t="inlineStr">
@@ -11036,14 +11036,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-12-12</t>
+        </is>
+      </c>
       <c r="I133" t="inlineStr">
         <is>
           <t xml:space="preserve">12/12/2025</t>
-        </is>
-      </c>
-      <c r="J133" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K133" t="inlineStr">
@@ -11118,14 +11118,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-12-12</t>
+        </is>
+      </c>
       <c r="I134" t="inlineStr">
         <is>
           <t xml:space="preserve">12/12/2025</t>
-        </is>
-      </c>
-      <c r="J134" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K134" t="inlineStr">
@@ -11200,14 +11200,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-10-07</t>
+        </is>
+      </c>
       <c r="I135" t="inlineStr">
         <is>
           <t xml:space="preserve">7/10/2025</t>
-        </is>
-      </c>
-      <c r="J135" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K135" t="inlineStr">
@@ -11446,14 +11446,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-06-12</t>
+        </is>
+      </c>
       <c r="I138" t="inlineStr">
         <is>
           <t xml:space="preserve">12/6/2026</t>
-        </is>
-      </c>
-      <c r="J138" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K138" t="inlineStr">
@@ -11528,14 +11528,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-06-12</t>
+        </is>
+      </c>
       <c r="I139" t="inlineStr">
         <is>
           <t xml:space="preserve">12/6/2026</t>
-        </is>
-      </c>
-      <c r="J139" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K139" t="inlineStr">
@@ -11610,14 +11610,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-06-12</t>
+        </is>
+      </c>
       <c r="I140" t="inlineStr">
         <is>
           <t xml:space="preserve">12/6/2026</t>
-        </is>
-      </c>
-      <c r="J140" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K140" t="inlineStr">
@@ -11692,14 +11692,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-06-12</t>
+        </is>
+      </c>
       <c r="I141" t="inlineStr">
         <is>
           <t xml:space="preserve">12/6/2026</t>
-        </is>
-      </c>
-      <c r="J141" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K141" t="inlineStr">
@@ -11774,14 +11774,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-06-12</t>
+        </is>
+      </c>
       <c r="I142" t="inlineStr">
         <is>
           <t xml:space="preserve">12/6/2026</t>
-        </is>
-      </c>
-      <c r="J142" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K142" t="inlineStr">
@@ -11856,14 +11856,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-06-12</t>
+        </is>
+      </c>
       <c r="I143" t="inlineStr">
         <is>
           <t xml:space="preserve">12/6/2026</t>
-        </is>
-      </c>
-      <c r="J143" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K143" t="inlineStr">
@@ -11938,14 +11938,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-10</t>
+        </is>
+      </c>
       <c r="I144" t="inlineStr">
         <is>
           <t xml:space="preserve">10/3/2026</t>
-        </is>
-      </c>
-      <c r="J144" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K144" t="inlineStr">
@@ -13347,14 +13347,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-07-03</t>
+        </is>
+      </c>
       <c r="I161" t="inlineStr">
         <is>
           <t xml:space="preserve">3/7/2025</t>
-        </is>
-      </c>
-      <c r="J161" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K161" t="inlineStr">
@@ -13439,14 +13439,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-07-03</t>
+        </is>
+      </c>
       <c r="I162" t="inlineStr">
         <is>
           <t xml:space="preserve">3/7/2025</t>
-        </is>
-      </c>
-      <c r="J162" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K162" t="inlineStr">
@@ -14177,14 +14177,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-08-11</t>
+        </is>
+      </c>
       <c r="I171" t="inlineStr">
         <is>
           <t xml:space="preserve">11/8/2025</t>
-        </is>
-      </c>
-      <c r="J171" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K171" t="inlineStr">
@@ -14341,14 +14341,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H173" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-06-01</t>
+        </is>
+      </c>
       <c r="I173" t="inlineStr">
         <is>
           <t xml:space="preserve">1/6/2026</t>
-        </is>
-      </c>
-      <c r="J173" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K173" t="inlineStr">
@@ -14423,14 +14423,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-06-01</t>
+        </is>
+      </c>
       <c r="I174" t="inlineStr">
         <is>
           <t xml:space="preserve">1/6/2026</t>
-        </is>
-      </c>
-      <c r="J174" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K174" t="inlineStr">
@@ -14505,14 +14505,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H175" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-05-06</t>
+        </is>
+      </c>
       <c r="I175" t="inlineStr">
         <is>
           <t xml:space="preserve">6/5/2026</t>
-        </is>
-      </c>
-      <c r="J175" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K175" t="inlineStr">
@@ -14587,14 +14587,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-05-06</t>
+        </is>
+      </c>
       <c r="I176" t="inlineStr">
         <is>
           <t xml:space="preserve">6/5/2026</t>
-        </is>
-      </c>
-      <c r="J176" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K176" t="inlineStr">
@@ -14669,14 +14669,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-05-06</t>
+        </is>
+      </c>
       <c r="I177" t="inlineStr">
         <is>
           <t xml:space="preserve">6/5/2026</t>
-        </is>
-      </c>
-      <c r="J177" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K177" t="inlineStr">
@@ -14751,14 +14751,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-06-01</t>
+        </is>
+      </c>
       <c r="I178" t="inlineStr">
         <is>
           <t xml:space="preserve">1/6/2026</t>
-        </is>
-      </c>
-      <c r="J178" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K178" t="inlineStr">
@@ -14833,14 +14833,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H179" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-06-01</t>
+        </is>
+      </c>
       <c r="I179" t="inlineStr">
         <is>
           <t xml:space="preserve">1/6/2026</t>
-        </is>
-      </c>
-      <c r="J179" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K179" t="inlineStr">
@@ -15775,14 +15775,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-07-03</t>
+        </is>
+      </c>
       <c r="I190" t="inlineStr">
         <is>
           <t xml:space="preserve">3/7/2025</t>
-        </is>
-      </c>
-      <c r="J190" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K190" t="inlineStr">
@@ -15857,14 +15857,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
+      <c r="H191" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-07-03</t>
+        </is>
+      </c>
       <c r="I191" t="inlineStr">
         <is>
           <t xml:space="preserve">3/7/2025</t>
-        </is>
-      </c>
-      <c r="J191" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K191" t="inlineStr">
@@ -16103,14 +16103,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
+      <c r="H194" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-06-02</t>
+        </is>
+      </c>
       <c r="I194" t="inlineStr">
         <is>
           <t xml:space="preserve">2/6/2025</t>
-        </is>
-      </c>
-      <c r="J194" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K194" t="inlineStr">
@@ -16185,14 +16185,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
+      <c r="H195" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-07-03</t>
+        </is>
+      </c>
       <c r="I195" t="inlineStr">
         <is>
           <t xml:space="preserve">3/7/2025</t>
-        </is>
-      </c>
-      <c r="J195" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K195" t="inlineStr">
@@ -16513,14 +16513,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H199" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-11-04</t>
+        </is>
+      </c>
       <c r="I199" t="inlineStr">
         <is>
           <t xml:space="preserve">4/11/2025</t>
-        </is>
-      </c>
-      <c r="J199" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K199" t="inlineStr">
@@ -16677,14 +16677,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H201" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-11-04</t>
+        </is>
+      </c>
       <c r="I201" t="inlineStr">
         <is>
           <t xml:space="preserve">4/11/2025</t>
-        </is>
-      </c>
-      <c r="J201" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K201" t="inlineStr">
@@ -17753,14 +17753,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H214" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-06-04</t>
+        </is>
+      </c>
       <c r="I214" t="inlineStr">
         <is>
           <t xml:space="preserve">4/6/2026</t>
-        </is>
-      </c>
-      <c r="J214" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K214" t="inlineStr">
@@ -17845,14 +17845,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H215" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-06-04</t>
+        </is>
+      </c>
       <c r="I215" t="inlineStr">
         <is>
           <t xml:space="preserve">4/6/2026</t>
-        </is>
-      </c>
-      <c r="J215" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K215" t="inlineStr">
@@ -18593,14 +18593,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H224" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-01-05</t>
+        </is>
+      </c>
       <c r="I224" t="inlineStr">
         <is>
           <t xml:space="preserve">5/1/2024</t>
-        </is>
-      </c>
-      <c r="J224" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K224" t="inlineStr">
@@ -18921,14 +18921,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H228" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-04-05</t>
+        </is>
+      </c>
       <c r="I228" t="inlineStr">
         <is>
           <t xml:space="preserve">5/4/2024</t>
-        </is>
-      </c>
-      <c r="J228" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K228" t="inlineStr">
@@ -19249,14 +19249,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H232" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-05-04</t>
+        </is>
+      </c>
       <c r="I232" t="inlineStr">
         <is>
           <t xml:space="preserve">4/5/2026</t>
-        </is>
-      </c>
-      <c r="J232" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K232" t="inlineStr">
@@ -19577,14 +19577,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H236" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-05</t>
+        </is>
+      </c>
       <c r="I236" t="inlineStr">
         <is>
           <t xml:space="preserve">5/3/2026</t>
-        </is>
-      </c>
-      <c r="J236" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K236" t="inlineStr">
@@ -19659,14 +19659,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H237" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-10</t>
+        </is>
+      </c>
       <c r="I237" t="inlineStr">
         <is>
           <t xml:space="preserve">10/8/2026</t>
-        </is>
-      </c>
-      <c r="J237" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K237" t="inlineStr">
@@ -19741,14 +19741,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H238" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-10</t>
+        </is>
+      </c>
       <c r="I238" t="inlineStr">
         <is>
           <t xml:space="preserve">10/8/2026</t>
-        </is>
-      </c>
-      <c r="J238" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K238" t="inlineStr">
@@ -19823,14 +19823,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H239" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-10</t>
+        </is>
+      </c>
       <c r="I239" t="inlineStr">
         <is>
           <t xml:space="preserve">10/8/2026</t>
-        </is>
-      </c>
-      <c r="J239" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K239" t="inlineStr">
@@ -20141,14 +20141,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H243" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-11-06</t>
+        </is>
+      </c>
       <c r="I243" t="inlineStr">
         <is>
           <t xml:space="preserve">6/11/2025</t>
-        </is>
-      </c>
-      <c r="J243" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K243" t="inlineStr">
@@ -20305,14 +20305,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H245" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-11-06</t>
+        </is>
+      </c>
       <c r="I245" t="inlineStr">
         <is>
           <t xml:space="preserve">6/11/2025</t>
-        </is>
-      </c>
-      <c r="J245" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K245" t="inlineStr">
@@ -20464,14 +20464,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H247" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-12-12</t>
+        </is>
+      </c>
       <c r="I247" t="inlineStr">
         <is>
           <t xml:space="preserve">12/12/2025</t>
-        </is>
-      </c>
-      <c r="J247" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K247" t="inlineStr">
@@ -20546,14 +20546,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H248" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-12-12</t>
+        </is>
+      </c>
       <c r="I248" t="inlineStr">
         <is>
           <t xml:space="preserve">12/12/2025</t>
-        </is>
-      </c>
-      <c r="J248" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K248" t="inlineStr">
@@ -20628,14 +20628,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H249" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-12-12</t>
+        </is>
+      </c>
       <c r="I249" t="inlineStr">
         <is>
           <t xml:space="preserve">12/12/2025</t>
-        </is>
-      </c>
-      <c r="J249" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K249" t="inlineStr">
@@ -20710,14 +20710,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H250" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-12-12</t>
+        </is>
+      </c>
       <c r="I250" t="inlineStr">
         <is>
           <t xml:space="preserve">12/12/2025</t>
-        </is>
-      </c>
-      <c r="J250" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K250" t="inlineStr">
@@ -20874,14 +20874,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H252" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-12-11</t>
+        </is>
+      </c>
       <c r="I252" t="inlineStr">
         <is>
           <t xml:space="preserve">11/12/2025</t>
-        </is>
-      </c>
-      <c r="J252" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K252" t="inlineStr">
@@ -21120,14 +21120,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H255" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-12-05</t>
+        </is>
+      </c>
       <c r="I255" t="inlineStr">
         <is>
           <t xml:space="preserve">5/12/2025</t>
-        </is>
-      </c>
-      <c r="J255" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K255" t="inlineStr">
@@ -21202,14 +21202,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H256" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-11-10</t>
+        </is>
+      </c>
       <c r="I256" t="inlineStr">
         <is>
           <t xml:space="preserve">10/11/2025</t>
-        </is>
-      </c>
-      <c r="J256" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K256" t="inlineStr">
@@ -21284,14 +21284,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H257" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-10</t>
+        </is>
+      </c>
       <c r="I257" t="inlineStr">
         <is>
           <t xml:space="preserve">10/8/2026</t>
-        </is>
-      </c>
-      <c r="J257" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K257" t="inlineStr">
@@ -21366,14 +21366,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H258" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-10</t>
+        </is>
+      </c>
       <c r="I258" t="inlineStr">
         <is>
           <t xml:space="preserve">10/8/2026</t>
-        </is>
-      </c>
-      <c r="J258" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K258" t="inlineStr">
@@ -21448,14 +21448,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H259" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-10</t>
+        </is>
+      </c>
       <c r="I259" t="inlineStr">
         <is>
           <t xml:space="preserve">10/8/2026</t>
-        </is>
-      </c>
-      <c r="J259" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K259" t="inlineStr">
@@ -21530,14 +21530,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H260" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-10</t>
+        </is>
+      </c>
       <c r="I260" t="inlineStr">
         <is>
           <t xml:space="preserve">10/8/2026</t>
-        </is>
-      </c>
-      <c r="J260" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K260" t="inlineStr">
@@ -21612,14 +21612,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H261" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-08-10</t>
+        </is>
+      </c>
       <c r="I261" t="inlineStr">
         <is>
           <t xml:space="preserve">10/8/2026</t>
-        </is>
-      </c>
-      <c r="J261" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K261" t="inlineStr">
@@ -21694,14 +21694,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
+      <c r="H262" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-12-02</t>
+        </is>
+      </c>
       <c r="I262" t="inlineStr">
         <is>
           <t xml:space="preserve">2/12/2025</t>
-        </is>
-      </c>
-      <c r="J262" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K262" t="inlineStr">
@@ -21776,14 +21776,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H263" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-12-04</t>
+        </is>
+      </c>
       <c r="I263" t="inlineStr">
         <is>
           <t xml:space="preserve">4/12/2025</t>
-        </is>
-      </c>
-      <c r="J263" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K263" t="inlineStr">
@@ -21858,14 +21858,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H264" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-12-04</t>
+        </is>
+      </c>
       <c r="I264" t="inlineStr">
         <is>
           <t xml:space="preserve">4/12/2025</t>
-        </is>
-      </c>
-      <c r="J264" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K264" t="inlineStr">
@@ -21940,14 +21940,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
+      <c r="H265" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-12-05</t>
+        </is>
+      </c>
       <c r="I265" t="inlineStr">
         <is>
           <t xml:space="preserve">5/12/2025</t>
-        </is>
-      </c>
-      <c r="J265" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K265" t="inlineStr">
@@ -22022,14 +22022,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
+      <c r="H266" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-12-02</t>
+        </is>
+      </c>
       <c r="I266" t="inlineStr">
         <is>
           <t xml:space="preserve">2/12/2025</t>
-        </is>
-      </c>
-      <c r="J266" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K266" t="inlineStr">
@@ -22104,14 +22104,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
+      <c r="H267" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-12-02</t>
+        </is>
+      </c>
       <c r="I267" t="inlineStr">
         <is>
           <t xml:space="preserve">2/12/2025</t>
-        </is>
-      </c>
-      <c r="J267" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K267" t="inlineStr">
@@ -22842,14 +22842,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H276" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-01-02</t>
+        </is>
+      </c>
       <c r="I276" t="inlineStr">
         <is>
           <t xml:space="preserve">2/1/2026</t>
-        </is>
-      </c>
-      <c r="J276" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K276" t="inlineStr">
@@ -22924,14 +22924,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H277" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-01-02</t>
+        </is>
+      </c>
       <c r="I277" t="inlineStr">
         <is>
           <t xml:space="preserve">2/1/2026</t>
-        </is>
-      </c>
-      <c r="J277" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K277" t="inlineStr">
@@ -23006,14 +23006,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H278" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-01-02</t>
+        </is>
+      </c>
       <c r="I278" t="inlineStr">
         <is>
           <t xml:space="preserve">2/1/2026</t>
-        </is>
-      </c>
-      <c r="J278" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K278" t="inlineStr">
@@ -23088,14 +23088,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H279" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-01-08</t>
+        </is>
+      </c>
       <c r="I279" t="inlineStr">
         <is>
           <t xml:space="preserve">8/1/2026</t>
-        </is>
-      </c>
-      <c r="J279" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K279" t="inlineStr">
@@ -23580,14 +23580,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H285" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-01-08</t>
+        </is>
+      </c>
       <c r="I285" t="inlineStr">
         <is>
           <t xml:space="preserve">8/1/2026</t>
-        </is>
-      </c>
-      <c r="J285" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K285" t="inlineStr">
@@ -24149,14 +24149,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H292" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-01-05</t>
+        </is>
+      </c>
       <c r="I292" t="inlineStr">
         <is>
           <t xml:space="preserve">5/1/2026</t>
-        </is>
-      </c>
-      <c r="J292" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K292" t="inlineStr">
@@ -24477,14 +24477,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H296" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-05-04</t>
+        </is>
+      </c>
       <c r="I296" t="inlineStr">
         <is>
           <t xml:space="preserve">4/5/2026</t>
-        </is>
-      </c>
-      <c r="J296" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K296" t="inlineStr">
@@ -24559,14 +24559,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H297" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-05-04</t>
+        </is>
+      </c>
       <c r="I297" t="inlineStr">
         <is>
           <t xml:space="preserve">4/5/2026</t>
-        </is>
-      </c>
-      <c r="J297" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K297" t="inlineStr">
@@ -24641,14 +24641,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H298" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-01-08</t>
+        </is>
+      </c>
       <c r="I298" t="inlineStr">
         <is>
           <t xml:space="preserve">8/1/2026</t>
-        </is>
-      </c>
-      <c r="J298" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K298" t="inlineStr">
@@ -24723,14 +24723,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H299" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-01-08</t>
+        </is>
+      </c>
       <c r="I299" t="inlineStr">
         <is>
           <t xml:space="preserve">8/1/2026</t>
-        </is>
-      </c>
-      <c r="J299" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K299" t="inlineStr">
@@ -24805,14 +24805,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H300" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-01-08</t>
+        </is>
+      </c>
       <c r="I300" t="inlineStr">
         <is>
           <t xml:space="preserve">8/1/2026</t>
-        </is>
-      </c>
-      <c r="J300" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K300" t="inlineStr">
@@ -24887,14 +24887,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H301" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-01-08</t>
+        </is>
+      </c>
       <c r="I301" t="inlineStr">
         <is>
           <t xml:space="preserve">8/1/2026</t>
-        </is>
-      </c>
-      <c r="J301" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K301" t="inlineStr">
@@ -24969,14 +24969,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H302" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-01-08</t>
+        </is>
+      </c>
       <c r="I302" t="inlineStr">
         <is>
           <t xml:space="preserve">8/1/2026</t>
-        </is>
-      </c>
-      <c r="J302" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K302" t="inlineStr">
@@ -25297,14 +25297,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H306" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-05-05</t>
+        </is>
+      </c>
       <c r="I306" t="inlineStr">
         <is>
           <t xml:space="preserve">5/5/2025</t>
-        </is>
-      </c>
-      <c r="J306" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K306" t="inlineStr">
@@ -25379,14 +25379,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H307" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-06-01</t>
+        </is>
+      </c>
       <c r="I307" t="inlineStr">
         <is>
           <t xml:space="preserve">1/6/2026</t>
-        </is>
-      </c>
-      <c r="J307" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K307" t="inlineStr">
@@ -25461,14 +25461,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H308" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-06-01</t>
+        </is>
+      </c>
       <c r="I308" t="inlineStr">
         <is>
           <t xml:space="preserve">1/6/2026</t>
-        </is>
-      </c>
-      <c r="J308" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K308" t="inlineStr">
@@ -25543,14 +25543,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H309" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-06-01</t>
+        </is>
+      </c>
       <c r="I309" t="inlineStr">
         <is>
           <t xml:space="preserve">1/6/2026</t>
-        </is>
-      </c>
-      <c r="J309" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K309" t="inlineStr">
@@ -25625,14 +25625,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H310" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-06-01</t>
+        </is>
+      </c>
       <c r="I310" t="inlineStr">
         <is>
           <t xml:space="preserve">1/6/2026</t>
-        </is>
-      </c>
-      <c r="J310" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K310" t="inlineStr">
@@ -26035,14 +26035,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H315" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-05-02</t>
+        </is>
+      </c>
       <c r="I315" t="inlineStr">
         <is>
           <t xml:space="preserve">2/5/2025</t>
-        </is>
-      </c>
-      <c r="J315" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K315" t="inlineStr">
@@ -26117,14 +26117,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H316" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-05-04</t>
+        </is>
+      </c>
       <c r="I316" t="inlineStr">
         <is>
           <t xml:space="preserve">4/5/2026</t>
-        </is>
-      </c>
-      <c r="J316" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K316" t="inlineStr">
@@ -26199,14 +26199,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H317" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-05-04</t>
+        </is>
+      </c>
       <c r="I317" t="inlineStr">
         <is>
           <t xml:space="preserve">4/5/2026</t>
-        </is>
-      </c>
-      <c r="J317" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K317" t="inlineStr">
@@ -26281,14 +26281,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H318" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-05-04</t>
+        </is>
+      </c>
       <c r="I318" t="inlineStr">
         <is>
           <t xml:space="preserve">4/5/2026</t>
-        </is>
-      </c>
-      <c r="J318" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K318" t="inlineStr">
@@ -26363,14 +26363,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H319" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-05-04</t>
+        </is>
+      </c>
       <c r="I319" t="inlineStr">
         <is>
           <t xml:space="preserve">4/5/2026</t>
-        </is>
-      </c>
-      <c r="J319" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K319" t="inlineStr">
@@ -26445,14 +26445,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H320" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-05-04</t>
+        </is>
+      </c>
       <c r="I320" t="inlineStr">
         <is>
           <t xml:space="preserve">4/5/2026</t>
-        </is>
-      </c>
-      <c r="J320" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K320" t="inlineStr">
@@ -26527,14 +26527,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H321" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-05-04</t>
+        </is>
+      </c>
       <c r="I321" t="inlineStr">
         <is>
           <t xml:space="preserve">4/5/2026</t>
-        </is>
-      </c>
-      <c r="J321" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K321" t="inlineStr">
@@ -26691,14 +26691,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H323" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-05-02</t>
+        </is>
+      </c>
       <c r="I323" t="inlineStr">
         <is>
           <t xml:space="preserve">2/5/2025</t>
-        </is>
-      </c>
-      <c r="J323" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K323" t="inlineStr">
@@ -27039,14 +27039,14 @@
           <t xml:space="preserve">relative</t>
         </is>
       </c>
+      <c r="H327" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-06-04</t>
+        </is>
+      </c>
       <c r="I327" t="inlineStr">
         <is>
           <t xml:space="preserve">4/6/2026</t>
-        </is>
-      </c>
-      <c r="J327" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K327" t="inlineStr">
@@ -27608,14 +27608,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H334" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-04-10</t>
+        </is>
+      </c>
       <c r="I334" t="inlineStr">
         <is>
           <t xml:space="preserve">10/4/2026</t>
-        </is>
-      </c>
-      <c r="J334" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K334" t="inlineStr">
@@ -27772,14 +27772,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H336" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-04-10</t>
+        </is>
+      </c>
       <c r="I336" t="inlineStr">
         <is>
           <t xml:space="preserve">10/4/2026</t>
-        </is>
-      </c>
-      <c r="J336" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K336" t="inlineStr">
@@ -27854,14 +27854,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H337" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-04-10</t>
+        </is>
+      </c>
       <c r="I337" t="inlineStr">
         <is>
           <t xml:space="preserve">10/4/2026</t>
-        </is>
-      </c>
-      <c r="J337" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K337" t="inlineStr">
@@ -27936,14 +27936,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H338" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-04-10</t>
+        </is>
+      </c>
       <c r="I338" t="inlineStr">
         <is>
           <t xml:space="preserve">10/4/2026</t>
-        </is>
-      </c>
-      <c r="J338" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K338" t="inlineStr">
@@ -28018,14 +28018,14 @@
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
+      <c r="H339" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-02-10</t>
+        </is>
+      </c>
       <c r="I339" t="inlineStr">
         <is>
           <t xml:space="preserve">10/2/2026</t>
-        </is>
-      </c>
-      <c r="J339" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K339" t="inlineStr">
@@ -28182,14 +28182,14 @@
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
+      <c r="H341" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-02-06</t>
+        </is>
+      </c>
       <c r="I341" t="inlineStr">
         <is>
           <t xml:space="preserve">6/2/2026</t>
-        </is>
-      </c>
-      <c r="J341" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="K341" t="inlineStr">

</xml_diff>

<commit_message>
Edit LnCapCASPEX no select E from Umut iphone cell stocks
</commit_message>
<xml_diff>
--- a/cellstocks/cell-stocks.xlsx
+++ b/cellstocks/cell-stocks.xlsx
@@ -26785,12 +26785,12 @@
       </c>
       <c r="F324" t="inlineStr">
         <is>
-          <t xml:space="preserve">p45769</t>
+          <t xml:space="preserve">p?</t>
         </is>
       </c>
       <c r="G324" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">unknown</t>
         </is>
       </c>
       <c r="J324" t="inlineStr">

</xml_diff>